<commit_message>
Add contact form, test mode page, and admin/award route enhancements
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testing/Amusement_Testing_Plan.xlsx
+++ b/testing/Amusement_Testing_Plan.xlsx
@@ -6,10 +6,12 @@
     <sheet name="Base Rates" sheetId="1" r:id="rId1"/>
     <sheet name="Penalty Rates" sheetId="2" r:id="rId2"/>
     <sheet name="Overtime" sheetId="3" r:id="rId3"/>
-    <sheet name="Min Engagement" sheetId="4" r:id="rId4"/>
-    <sheet name="Allowances" sheetId="5" r:id="rId5"/>
-    <sheet name="Superannuation" sheetId="6" r:id="rId6"/>
-    <sheet name="Regression" sheetId="7" r:id="rId7"/>
+    <sheet name="CDO" sheetId="4" r:id="rId4"/>
+    <sheet name="CWO" sheetId="5" r:id="rId5"/>
+    <sheet name="Min Engagement" sheetId="6" r:id="rId6"/>
+    <sheet name="Allowances" sheetId="7" r:id="rId7"/>
+    <sheet name="Superannuation" sheetId="8" r:id="rId8"/>
+    <sheet name="Regression" sheetId="9" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
@@ -1148,36 +1150,36 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ME-01</v>
+        <v>CDO-01</v>
       </c>
       <c r="B2" t="str">
-        <v>62.38</v>
+        <v>yes</v>
       </c>
       <c r="C2" t="str">
-        <v>62.38</v>
+        <v>yes</v>
       </c>
       <c r="D2" t="str">
         <v>PASS</v>
       </c>
       <c r="E2" t="str">
-        <v>Casual 1hr → 2hr min</v>
+        <v>Casual 13.5hr triggers daily OT (OT=$28.07)</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ME-02</v>
+        <v>CDO-02</v>
       </c>
       <c r="B3" t="str">
-        <v>87.33</v>
+        <v>0</v>
       </c>
       <c r="C3" t="str">
-        <v>87.33</v>
+        <v>0</v>
       </c>
       <c r="D3" t="str">
         <v>PASS</v>
       </c>
       <c r="E3" t="str">
-        <v>Casual Sunday 1hr → 2hr min @1.40×</v>
+        <v>Casual 9hr = no daily OT (under 10hr threshold)</v>
       </c>
     </row>
   </sheetData>
@@ -1189,7 +1191,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1217,92 +1219,24 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>AL-01</v>
+        <v>CWO-01</v>
       </c>
       <c r="B2" t="str">
-        <v>0.56</v>
+        <v>yes</v>
       </c>
       <c r="C2" t="str">
-        <v>0.56</v>
+        <v>yes</v>
       </c>
       <c r="D2" t="str">
         <v>PASS</v>
       </c>
       <c r="E2" t="str">
-        <v>First aid per hour</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>AL-02</v>
-      </c>
-      <c r="B3" t="str">
-        <v>14.62</v>
-      </c>
-      <c r="C3" t="str">
-        <v>14.62</v>
-      </c>
-      <c r="D3" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Meal allowance</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>AL-04</v>
-      </c>
-      <c r="B4" t="str">
-        <v>15.83</v>
-      </c>
-      <c r="C4" t="str">
-        <v>15.83</v>
-      </c>
-      <c r="D4" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Tool tradesperson weekly</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>AL-05</v>
-      </c>
-      <c r="B5" t="str">
-        <v>0.84</v>
-      </c>
-      <c r="C5" t="str">
-        <v>0.84</v>
-      </c>
-      <c r="D5" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Tractor plant per hour</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>AL-03</v>
-      </c>
-      <c r="B6" t="str">
-        <v>0.98</v>
-      </c>
-      <c r="C6" t="str">
-        <v>0.98</v>
-      </c>
-      <c r="D6" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Vehicle per km</v>
+        <v>Casual 40hr week triggers weekly OT (OT=$12.48)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1337,36 +1271,36 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>SU-01</v>
+        <v>ME-01</v>
       </c>
       <c r="B2" t="str">
-        <v>24.35</v>
+        <v>62.38</v>
       </c>
       <c r="C2" t="str">
-        <v>24.35</v>
+        <v>62.38</v>
       </c>
       <c r="D2" t="str">
         <v>PASS</v>
       </c>
       <c r="E2" t="str">
-        <v>Super on 7.6hr weekday (daily threshold)</v>
+        <v>Casual 1hr → 2hr min</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>SU-02</v>
+        <v>ME-02</v>
       </c>
       <c r="B3" t="str">
-        <v>0.12</v>
+        <v>87.33</v>
       </c>
       <c r="C3" t="str">
-        <v>0.12</v>
+        <v>87.33</v>
       </c>
       <c r="D3" t="str">
         <v>PASS</v>
       </c>
       <c r="E3" t="str">
-        <v>SGC 12%</v>
+        <v>Casual Sunday 1hr → 2hr min @1.40×</v>
       </c>
     </row>
   </sheetData>
@@ -1377,6 +1311,126 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E6"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="60.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Test ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Expected</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Actual Output</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Result</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>AL-01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>0.56</v>
+      </c>
+      <c r="C2" t="str">
+        <v>0.56</v>
+      </c>
+      <c r="D2" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="E2" t="str">
+        <v>First aid per hour</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>AL-02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>14.62</v>
+      </c>
+      <c r="C3" t="str">
+        <v>14.62</v>
+      </c>
+      <c r="D3" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Meal allowance</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>AL-04</v>
+      </c>
+      <c r="B4" t="str">
+        <v>15.83</v>
+      </c>
+      <c r="C4" t="str">
+        <v>15.83</v>
+      </c>
+      <c r="D4" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Tool tradesperson weekly</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>AL-05</v>
+      </c>
+      <c r="B5" t="str">
+        <v>0.84</v>
+      </c>
+      <c r="C5" t="str">
+        <v>0.84</v>
+      </c>
+      <c r="D5" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Tractor plant per hour</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>AL-03</v>
+      </c>
+      <c r="B6" t="str">
+        <v>0.98</v>
+      </c>
+      <c r="C6" t="str">
+        <v>0.98</v>
+      </c>
+      <c r="D6" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Vehicle per km</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E3"/>
   <cols>
@@ -1406,6 +1460,75 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>SU-01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>24.35</v>
+      </c>
+      <c r="C2" t="str">
+        <v>24.35</v>
+      </c>
+      <c r="D2" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Super on 7.6hr weekday (daily threshold)</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>SU-02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>0.12</v>
+      </c>
+      <c r="C3" t="str">
+        <v>0.12</v>
+      </c>
+      <c r="D3" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="E3" t="str">
+        <v>SGC 12%</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E3"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="60.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Test ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Expected</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Actual Output</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Result</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
         <v>RT-01</v>
       </c>
       <c r="B2" t="str">

</xml_diff>